<commit_message>
feat: auto-order admission numbers, enforce alphabetical sorting portal-wide, and replace manual subjects with CSV allocation
</commit_message>
<xml_diff>
--- a/public/templates/teacher_upload_template.xlsx
+++ b/public/templates/teacher_upload_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,6 +421,9 @@
       <c r="G1" t="str">
         <v>qualification</v>
       </c>
+      <c r="H1" t="str">
+        <v>subjects</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -442,12 +445,15 @@
         <v>2024-06-01</v>
       </c>
       <c r="G2" t="str">
-        <v>M.Sc, B.Ed</v>
+        <v>M.Sc B.Ed</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Science</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>